<commit_message>
feat: Weekly Crush sheet in Excel (live formulas) + standalone template
- yellow weekly price rows; placement, marketing date, contract, prices and every cost
  line are formulas over the workbook's named inputs (same ration/costs/hedges/debt)
- LibreOffice parity test vs crush_table (futures and cash corn, Dec->Feb roll)
- app download and W2F_Projection.xlsx include the crush; template uses the contract rule

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTSCZNmEoT9CgCPoTHxFfB
</commit_message>
<xml_diff>
--- a/W2F_Projection.xlsx
+++ b/W2F_Projection.xlsx
@@ -14,66 +14,104 @@
     <sheet name="Marketing" sheetId="5" r:id="rId5"/>
     <sheet name="Market Data" sheetId="6" r:id="rId6"/>
     <sheet name="Costs" sheetId="7" r:id="rId7"/>
+    <sheet name="Weekly Crush" sheetId="8" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="AvgDays">SUMPRODUCT(Marketing!$A$2:$A$9,Marketing!$B$2:$B$9)/100</definedName>
-    <definedName name="BarnDays">Inputs!$C$54</definedName>
-    <definedName name="BarnDowntime">Inputs!$C$28</definedName>
-    <definedName name="BarnMode">Inputs!$C$27</definedName>
-    <definedName name="BarnPerPig">Inputs!$C$29</definedName>
-    <definedName name="BarnRent">Inputs!$C$48</definedName>
+    <definedName name="BarnDays">Inputs!$C$72</definedName>
+    <definedName name="BarnDowntime">Inputs!$C$36</definedName>
+    <definedName name="BarnMode">Inputs!$C$35</definedName>
+    <definedName name="BarnPerPig">Inputs!$C$37</definedName>
+    <definedName name="BarnRent">Inputs!$C$66</definedName>
     <definedName name="BasisByPeriod">'Market Data'!$F$3:$F$26</definedName>
     <definedName name="CarcassCwt">SUMPRODUCT(Marketing!$K$2:$K$9,Marketing!$L$2:$L$9)/100</definedName>
-    <definedName name="CheckoffCost">Costs!$B$11</definedName>
-    <definedName name="CheckoffPct">Inputs!$C$41</definedName>
-    <definedName name="CornBasis">Inputs!$C$45</definedName>
-    <definedName name="CornCash">Inputs!$C$50</definedName>
-    <definedName name="CornFutures">Inputs!$C$22</definedName>
-    <definedName name="DdgsPrice">Inputs!$C$47</definedName>
-    <definedName name="DeadFeedShare">Inputs!$C$10</definedName>
+    <definedName name="CheckoffCost">Costs!$B$14</definedName>
+    <definedName name="CheckoffPct">Inputs!$C$53</definedName>
+    <definedName name="CornBasis">Inputs!$C$63</definedName>
+    <definedName name="CornCarry">Inputs!$C$28</definedName>
+    <definedName name="CornCash">Inputs!$C$68</definedName>
+    <definedName name="CornFutures">Inputs!$C$25</definedName>
+    <definedName name="CornHedged">Inputs!$C$30</definedName>
+    <definedName name="CornHedgePct">Inputs!$C$29</definedName>
+    <definedName name="CostBarn">Costs!$B$4</definedName>
+    <definedName name="CostCheckoff">Costs!$B$14</definedName>
+    <definedName name="CostFeed">Costs!$B$3</definedName>
+    <definedName name="CostGA">Costs!$B$10</definedName>
+    <definedName name="CostInsMisc">Costs!$B$9</definedName>
+    <definedName name="CostInterest">Costs!$B$13</definedName>
+    <definedName name="CostLabor">Costs!$B$5</definedName>
+    <definedName name="CostMortality">Costs!$B$11</definedName>
+    <definedName name="CostOther">Costs!$B$12</definedName>
+    <definedName name="CostPigs">Costs!$B$2</definedName>
+    <definedName name="CostTrucking">Costs!$B$8</definedName>
+    <definedName name="CostUtilities">Costs!$B$7</definedName>
+    <definedName name="CostVet">Costs!$B$6</definedName>
+    <definedName name="CrCornCash">'Weekly Crush'!$B$7</definedName>
+    <definedName name="CrDays">'Weekly Crush'!$B$5</definedName>
+    <definedName name="CrLag">'Weekly Crush'!$B$4</definedName>
+    <definedName name="CrWeight">'Weekly Crush'!$B$6</definedName>
+    <definedName name="DdgsPrice">Inputs!$C$65</definedName>
+    <definedName name="DeadFeedShare">Inputs!$C$12</definedName>
+    <definedName name="FeedCornBu">Feed!$I$14</definedName>
     <definedName name="FeedCost">Feed!$M$14</definedName>
-    <definedName name="FeedMill">Inputs!$C$24</definedName>
+    <definedName name="FeedDdgsTons">Feed!$K$14</definedName>
+    <definedName name="FeedMill">Inputs!$C$27</definedName>
+    <definedName name="FeedOtherUsd">SUMPRODUCT(Feed!$L$2:$L$13,Feed!$G$2:$G$13)</definedName>
+    <definedName name="FeedSbmTons">Feed!$J$14</definedName>
     <definedName name="FeedTons">Feed!$H$14</definedName>
     <definedName name="FutContracts">'Market Data'!$A$3:$A$26</definedName>
     <definedName name="FutPrices">'Market Data'!$B$3:$B$26</definedName>
+    <definedName name="GA">Inputs!$C$45</definedName>
     <definedName name="GrossRevenue">Marketing!$M$10</definedName>
     <definedName name="HeadPlaced">Inputs!$C$6</definedName>
-    <definedName name="HeadSold">Inputs!$C$53</definedName>
-    <definedName name="InsMisc">Inputs!$C$36</definedName>
-    <definedName name="InterestPct">Inputs!$C$37</definedName>
-    <definedName name="LaborHours">Inputs!$C$31</definedName>
-    <definedName name="LaborMode">Inputs!$C$30</definedName>
-    <definedName name="LaborPerPig">Inputs!$C$32</definedName>
-    <definedName name="LaborWage">Inputs!$C$49</definedName>
+    <definedName name="HeadSold">Inputs!$C$71</definedName>
+    <definedName name="HogHedged">Inputs!$C$55</definedName>
+    <definedName name="HogHedgePct">Inputs!$C$54</definedName>
+    <definedName name="InsMisc">Inputs!$C$44</definedName>
+    <definedName name="InterestMode">Inputs!$C$47</definedName>
+    <definedName name="InterestPct">Inputs!$C$49</definedName>
+    <definedName name="InterestPerPig">Inputs!$C$48</definedName>
+    <definedName name="LaborHours">Inputs!$C$39</definedName>
+    <definedName name="LaborMode">Inputs!$C$38</definedName>
+    <definedName name="LaborPerPig">Inputs!$C$40</definedName>
+    <definedName name="LaborWage">Inputs!$C$67</definedName>
     <definedName name="LiveCwt">SUMPRODUCT(Marketing!$K$2:$K$9,Marketing!$C$2:$C$9)/100</definedName>
-    <definedName name="Location">Inputs!$C$12</definedName>
-    <definedName name="LocRow">Inputs!$C$44</definedName>
-    <definedName name="MortalityPct">Inputs!$C$9</definedName>
-    <definedName name="PigsFed">Inputs!$C$55</definedName>
+    <definedName name="Location">Inputs!$C$14</definedName>
+    <definedName name="LocRow">Inputs!$C$62</definedName>
+    <definedName name="MortalityPct">Inputs!$C$10</definedName>
+    <definedName name="MortCost">Inputs!$C$11</definedName>
+    <definedName name="MortMode">Inputs!$C$9</definedName>
+    <definedName name="OtherSold">Inputs!$C$46</definedName>
+    <definedName name="PigsFed">Inputs!$C$73</definedName>
     <definedName name="PlacementDate">Inputs!$C$7</definedName>
-    <definedName name="Premium">Inputs!$C$40</definedName>
-    <definedName name="SbmBasis">Inputs!$C$46</definedName>
-    <definedName name="SbmCash">Inputs!$C$51</definedName>
-    <definedName name="SbmFutures">Inputs!$C$23</definedName>
-    <definedName name="TotalCost">Costs!$B$12</definedName>
-    <definedName name="Trucking">Inputs!$C$35</definedName>
-    <definedName name="Utilities">Inputs!$C$34</definedName>
-    <definedName name="VetMed">Inputs!$C$33</definedName>
-    <definedName name="WeanCash">Inputs!$C$16</definedName>
-    <definedName name="WeanFormula">Inputs!$C$17</definedName>
-    <definedName name="WeanFreight">Inputs!$C$19</definedName>
-    <definedName name="WeanManual">Inputs!$C$18</definedName>
-    <definedName name="WeanPrice">Inputs!$C$52</definedName>
-    <definedName name="WeanSource">Inputs!$C$15</definedName>
+    <definedName name="Premium">Inputs!$C$52</definedName>
+    <definedName name="Principal">Inputs!$C$58</definedName>
+    <definedName name="SbmBasis">Inputs!$C$64</definedName>
+    <definedName name="SbmCash">Inputs!$C$69</definedName>
+    <definedName name="SbmFutures">Inputs!$C$26</definedName>
+    <definedName name="SbmHedged">Inputs!$C$32</definedName>
+    <definedName name="SbmHedgePct">Inputs!$C$31</definedName>
+    <definedName name="TermInterest">Inputs!$C$59</definedName>
+    <definedName name="TotalCost">Costs!$B$15</definedName>
+    <definedName name="Trucking">Inputs!$C$43</definedName>
+    <definedName name="Utilities">Inputs!$C$42</definedName>
+    <definedName name="VetMed">Inputs!$C$41</definedName>
+    <definedName name="WeanAdder">Inputs!$C$20</definedName>
+    <definedName name="WeanCash">Inputs!$C$18</definedName>
+    <definedName name="WeanFormula">Inputs!$C$19</definedName>
+    <definedName name="WeanFreight">Inputs!$C$22</definedName>
+    <definedName name="WeanManual">Inputs!$C$21</definedName>
+    <definedName name="WeanPrice">Inputs!$C$70</definedName>
+    <definedName name="WeanSource">Inputs!$C$17</definedName>
     <definedName name="WeanWeight">Inputs!$C$8</definedName>
-    <definedName name="YieldPct">Inputs!$C$11</definedName>
+    <definedName name="YieldPct">Inputs!$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="265">
   <si>
     <t>Inputs — yellow cells are editable</t>
   </si>
@@ -102,12 +140,27 @@
     <t>lb</t>
   </si>
   <si>
+    <t>Mortality method</t>
+  </si>
+  <si>
+    <t>% of head</t>
+  </si>
+  <si>
+    <t>% of head = fewer pigs sold; $ per pig = flat death-loss charge</t>
+  </si>
+  <si>
     <t>Mortality (wean to market)</t>
   </si>
   <si>
     <t>%</t>
   </si>
   <si>
+    <t>Mortality charge if $ per pig</t>
+  </si>
+  <si>
+    <t>$/pig placed</t>
+  </si>
+  <si>
     <t>Feed eaten by a dead pig (share of full budget)</t>
   </si>
   <si>
@@ -159,6 +212,12 @@
     <t>Same report, formula purchases</t>
   </si>
   <si>
+    <t>Price adder over USDA</t>
+  </si>
+  <si>
+    <t>Your system's premium over the USDA price (not added to Manual)</t>
+  </si>
+  <si>
     <t>Manual weaned pig price</t>
   </si>
   <si>
@@ -183,6 +242,24 @@
     <t>Feed mill grind/mix/delivery</t>
   </si>
   <si>
+    <t>Corn carry / storage adder</t>
+  </si>
+  <si>
+    <t>Corn % hedged</t>
+  </si>
+  <si>
+    <t>Corn hedged/contracted cash price</t>
+  </si>
+  <si>
+    <t>All-in price on the hedged share</t>
+  </si>
+  <si>
+    <t>Soybean meal % hedged</t>
+  </si>
+  <si>
+    <t>Soybean meal hedged/contracted price</t>
+  </si>
+  <si>
     <t>Barn, labor and other</t>
   </si>
   <si>
@@ -243,6 +320,24 @@
     <t>Insurance / misc</t>
   </si>
   <si>
+    <t>G&amp;A</t>
+  </si>
+  <si>
+    <t>Other / (sales premiums)</t>
+  </si>
+  <si>
+    <t>Negative = premiums received</t>
+  </si>
+  <si>
+    <t>Interest method</t>
+  </si>
+  <si>
+    <t>annual rate</t>
+  </si>
+  <si>
+    <t>Interest if $ per pig</t>
+  </si>
+  <si>
     <t>Operating interest rate</t>
   </si>
   <si>
@@ -267,6 +362,24 @@
     <t>% of gross</t>
   </si>
   <si>
+    <t>Hogs % hedged</t>
+  </si>
+  <si>
+    <t>Hog hedged futures price</t>
+  </si>
+  <si>
+    <t>Futures locked on the hedged share; basis still applies</t>
+  </si>
+  <si>
+    <t>Debt service (below the operating margin)</t>
+  </si>
+  <si>
+    <t>Principal payment</t>
+  </si>
+  <si>
+    <t>Term interest payment</t>
+  </si>
+  <si>
     <t>From selected location (edit on Locations sheet)</t>
   </si>
   <si>
@@ -288,10 +401,10 @@
     <t>Labor wage $/hr</t>
   </si>
   <si>
-    <t>Corn cash price (futures + basis)</t>
-  </si>
-  <si>
-    <t>Soybean meal cash price (futures + basis)</t>
+    <t>Corn price paid (futures + basis + carry, blended with hedge)</t>
+  </si>
+  <si>
+    <t>Soybean meal price paid (futures + basis, blended with hedge)</t>
   </si>
   <si>
     <t>Weaned pig price used</t>
@@ -645,6 +758,12 @@
     <t>Utilities</t>
   </si>
   <si>
+    <t>Mortality ($/pig)</t>
+  </si>
+  <si>
+    <t>Other / (premiums)</t>
+  </si>
+  <si>
     <t>Interest</t>
   </si>
   <si>
@@ -672,6 +791,12 @@
     <t>Cost $/head sold</t>
   </si>
   <si>
+    <t>Debt service (principal + term interest)</t>
+  </si>
+  <si>
+    <t>Net $/head sold after debt service</t>
+  </si>
+  <si>
     <t>Breakeven $/cwt carcass</t>
   </si>
   <si>
@@ -690,16 +815,97 @@
     <t>Key prices</t>
   </si>
   <si>
-    <t>Corn cash $/bu (futures + basis)</t>
-  </si>
-  <si>
-    <t>Soybean meal cash $/ton</t>
+    <t>Corn $/bu paid (futures + basis + carry, hedge blend)</t>
+  </si>
+  <si>
+    <t>Soybean meal $/ton paid (hedge blend)</t>
   </si>
   <si>
     <t>Soybean meal basis $/ton</t>
   </si>
   <si>
     <t>Weaned pig $/head</t>
+  </si>
+  <si>
+    <t>Weekly Crush — margin per pig by weekly placement</t>
+  </si>
+  <si>
+    <t>Yellow cells are inputs. Costs, ration, hedges and debt come from the Inputs/Feed/Costs sheets.</t>
+  </si>
+  <si>
+    <t>Report → placement (days)</t>
+  </si>
+  <si>
+    <t>Days to average marketing</t>
+  </si>
+  <si>
+    <t>Sale weight (lb live)</t>
+  </si>
+  <si>
+    <t>Corn prices are cash (Yes/No)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>USDA report date</t>
+  </si>
+  <si>
+    <t>USDA weaned pig $/hd</t>
+  </si>
+  <si>
+    <t>Corn $/bu</t>
+  </si>
+  <si>
+    <t>Soybean meal $/ton</t>
+  </si>
+  <si>
+    <t>Lean hog futures $/cwt</t>
+  </si>
+  <si>
+    <t>Hog basis $/cwt</t>
+  </si>
+  <si>
+    <t>Avg marketing date</t>
+  </si>
+  <si>
+    <t>CME contract</t>
+  </si>
+  <si>
+    <t>Corn $/bu paid</t>
+  </si>
+  <si>
+    <t>Soybean meal $/ton paid</t>
+  </si>
+  <si>
+    <t>Revenue $/pig</t>
+  </si>
+  <si>
+    <t>Weaned pig $/pig</t>
+  </si>
+  <si>
+    <t>Feed $/pig</t>
+  </si>
+  <si>
+    <t>Barn / facilities $/pig</t>
+  </si>
+  <si>
+    <t>Other fixed costs $/pig</t>
+  </si>
+  <si>
+    <t>Interest $/pig</t>
+  </si>
+  <si>
+    <t>Checkoff $/pig</t>
+  </si>
+  <si>
+    <t>Cost of production $/pig</t>
+  </si>
+  <si>
+    <t>Margin $/pig</t>
+  </si>
+  <si>
+    <t>Margin after debt service $/pig</t>
   </si>
 </sst>
 </file>
@@ -712,8 +918,8 @@
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="#,##0.00"/>
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="@"/>
+    <numFmt numFmtId="169" formatCode="@"/>
+    <numFmt numFmtId="170" formatCode="0.00"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
   </numFmts>
   <fonts count="6">
@@ -851,7 +1057,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -872,6 +1078,9 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -933,9 +1142,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Costs!$A$2:$A$11</c:f>
+              <c:f>Costs!$A$2:$A$14</c:f>
               <c:strCache>
-                <c:ptCount val="10"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>Weaned pigs</c:v>
                 </c:pt>
@@ -961,9 +1170,18 @@
                   <c:v>Insurance / misc</c:v>
                 </c:pt>
                 <c:pt idx="8">
+                  <c:v>G&amp;A</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Mortality ($/pig)</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Other / (premiums)</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>Interest</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="12">
                   <c:v>Checkoff</c:v>
                 </c:pt>
               </c:strCache>
@@ -971,10 +1189,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Costs!$D$2:$D$11</c:f>
+              <c:f>Costs!$D$2:$D$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1003,6 +1221,15 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -1055,13 +1282,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1372,7 +1599,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:F17"/>
+  <dimension ref="B1:F19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -1385,7 +1612,7 @@
   <sheetData>
     <row r="1" spans="2:6">
       <c r="B1" s="1" t="s">
-        <v>193</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="2:6">
@@ -1396,14 +1623,14 @@
     </row>
     <row r="4" spans="2:6">
       <c r="B4" s="3" t="s">
-        <v>194</v>
+        <v>221</v>
       </c>
       <c r="C4" s="4">
         <f>GrossRevenue-TotalCost</f>
         <v>0</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
       <c r="F4" s="5">
         <f>(TotalCost-CheckoffCost)/(CarcassCwt*(1-CheckoffPct/100))</f>
@@ -1412,14 +1639,14 @@
     </row>
     <row r="5" spans="2:6">
       <c r="B5" s="3" t="s">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="C5" s="5">
         <f>(GrossRevenue-TotalCost)/HeadSold</f>
         <v>0</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="F5" s="5">
         <f>F4*YieldPct/100</f>
@@ -1428,14 +1655,14 @@
     </row>
     <row r="6" spans="2:6">
       <c r="B6" s="3" t="s">
-        <v>196</v>
+        <v>223</v>
       </c>
       <c r="C6" s="4">
         <f>GrossRevenue</f>
         <v>0</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="F6" s="5">
         <f>GrossRevenue/CarcassCwt</f>
@@ -1444,14 +1671,14 @@
     </row>
     <row r="7" spans="2:6">
       <c r="B7" s="3" t="s">
-        <v>192</v>
+        <v>219</v>
       </c>
       <c r="C7" s="4">
         <f>TotalCost</f>
         <v>0</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
       <c r="F7" s="5">
         <f>TotalCost/CarcassCwt</f>
@@ -1460,14 +1687,14 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" s="3" t="s">
-        <v>197</v>
+        <v>224</v>
       </c>
       <c r="C8" s="5">
         <f>GrossRevenue/HeadSold</f>
         <v>0</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="F8" s="6">
         <f>HeadSold</f>
@@ -1476,75 +1703,93 @@
     </row>
     <row r="9" spans="2:6">
       <c r="B9" s="3" t="s">
-        <v>198</v>
+        <v>225</v>
       </c>
       <c r="C9" s="5">
         <f>TotalCost/HeadSold</f>
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="F9" s="7">
         <f>IF(LiveCwt*100-HeadPlaced*WeanWeight&lt;=0,"n/a",FeedTons*2000/(LiveCwt*100-HeadPlaced*WeanWeight))</f>
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="2:6">
+      <c r="B10" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C10" s="4">
+        <f>HeadSold*(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="11" spans="2:6">
-      <c r="B11" s="8" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="12" spans="2:6">
-      <c r="B12" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="C12" s="5">
-        <f>CornCash</f>
+      <c r="B11" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="C11" s="5">
+        <f>(GrossRevenue-TotalCost)/HeadSold-(Principal+TermInterest)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="2:6">
-      <c r="B13" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="5">
-        <f>CornBasis</f>
-        <v>0</v>
+      <c r="B13" s="8" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="14" spans="2:6">
       <c r="B14" s="9" t="s">
-        <v>206</v>
+        <v>234</v>
       </c>
       <c r="C14" s="5">
-        <f>SbmCash</f>
+        <f>CornCash</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:6">
       <c r="B15" s="9" t="s">
-        <v>207</v>
+        <v>104</v>
       </c>
       <c r="C15" s="5">
-        <f>SbmBasis</f>
+        <f>CornBasis</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:6">
       <c r="B16" s="9" t="s">
-        <v>81</v>
+        <v>235</v>
       </c>
       <c r="C16" s="5">
-        <f>DdgsPrice</f>
+        <f>SbmCash</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:3">
       <c r="B17" s="9" t="s">
-        <v>208</v>
+        <v>236</v>
       </c>
       <c r="C17" s="5">
+        <f>SbmBasis</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C18" s="5">
+        <f>DdgsPrice</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="C19" s="5">
         <f>WeanPrice</f>
         <v>0</v>
       </c>
@@ -1561,7 +1806,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E55"/>
+  <dimension ref="B1:E73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -1626,95 +1871,91 @@
       <c r="B9" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="13">
-        <v>6.8</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C9" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="12">
-        <v>0.25</v>
+        <v>12</v>
+      </c>
+      <c r="C10" s="14">
+        <v>6.8</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="E10" s="2"/>
     </row>
     <row r="11" spans="2:5">
       <c r="B11" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="13">
-        <v>75</v>
+      <c r="C11" s="12">
+        <v>0</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E11" s="2"/>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="2"/>
       <c r="E12" s="2" t="s">
         <v>18</v>
       </c>
     </row>
+    <row r="13" spans="2:5">
+      <c r="B13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="14">
+        <v>75</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
     <row r="14" spans="2:5">
-      <c r="B14" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5">
-      <c r="B15" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="14" t="s">
+      <c r="B14" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2" t="s">
+      <c r="C14" s="13" t="s">
         <v>22</v>
       </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="16" spans="2:5">
-      <c r="B16" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="12">
-        <v>24.81</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="B16" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="12">
-        <v>24.81</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
         <v>27</v>
       </c>
@@ -1727,356 +1968,571 @@
         <v>24.81</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="2"/>
+        <v>29</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="12">
-        <v>1</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="12">
+        <v>0</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="21" spans="2:5">
-      <c r="B21" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="B21" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E21" s="2"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="9" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C22" s="12">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="12">
         <v>4.7425</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="2:5">
-      <c r="B23" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" s="12">
+      <c r="D25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="12">
         <v>357.1</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="2:5">
-      <c r="B24" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="12">
-        <v>15</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="26" spans="2:5">
-      <c r="B26" s="8" t="s">
-        <v>36</v>
-      </c>
+      <c r="D26" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E26" s="2"/>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" s="2"/>
+        <v>42</v>
+      </c>
+      <c r="C27" s="12">
+        <v>15</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="E27" s="2"/>
     </row>
     <row r="28" spans="2:5">
       <c r="B28" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="12">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C28" s="10">
-        <v>10</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>41</v>
-      </c>
+      <c r="E28" s="2"/>
     </row>
     <row r="29" spans="2:5">
       <c r="B29" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C29" s="12">
+        <v>44</v>
+      </c>
+      <c r="C29" s="14">
         <v>0</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="E29" s="2"/>
     </row>
     <row r="30" spans="2:5">
       <c r="B30" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C30" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="C30" s="12">
+        <v>0</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C31" s="12">
-        <v>0.2</v>
+        <v>47</v>
+      </c>
+      <c r="C31" s="14">
+        <v>0</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>48</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="E31" s="2"/>
     </row>
     <row r="32" spans="2:5">
       <c r="B32" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="12">
+        <v>0</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5">
+      <c r="B34" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C32" s="12">
-        <v>0</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E32" s="2"/>
-    </row>
-    <row r="33" spans="2:5">
-      <c r="B33" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="12">
-        <v>5</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E33" s="2"/>
-    </row>
-    <row r="34" spans="2:5">
-      <c r="B34" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="C34" s="12">
-        <v>4</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E34" s="2"/>
     </row>
     <row r="35" spans="2:5">
       <c r="B35" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C35" s="12">
-        <v>4</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>54</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D35" s="2"/>
       <c r="E35" s="2"/>
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="12">
-        <v>0.5</v>
+        <v>52</v>
+      </c>
+      <c r="C36" s="10">
+        <v>10</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E36" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" s="12">
+        <v>0</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="13">
-        <v>7.12</v>
-      </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="2:5">
+      <c r="B38" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="C38" s="13" t="s">
         <v>58</v>
       </c>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
     </row>
     <row r="39" spans="2:5">
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="9" t="s">
         <v>59</v>
+      </c>
+      <c r="C39" s="12">
+        <v>0.2</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C40" s="12">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E40" s="2"/>
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="C41" s="13">
-        <v>0.35</v>
+        <v>63</v>
+      </c>
+      <c r="C41" s="12">
+        <v>5</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E41" s="2"/>
     </row>
+    <row r="42" spans="2:5">
+      <c r="B42" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" s="12">
+        <v>4</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E42" s="2"/>
+    </row>
     <row r="43" spans="2:5">
-      <c r="B43" s="8" t="s">
-        <v>64</v>
-      </c>
+      <c r="B43" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C43" s="12">
+        <v>4</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E43" s="2"/>
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C44" s="6">
-        <f>MATCH(Location,Locations!$A$2:$A$61,0)</f>
-        <v>0</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="C44" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E44" s="2"/>
     </row>
     <row r="45" spans="2:5">
       <c r="B45" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="C45" s="7">
-        <f>INDEX(Locations!$C$2:$C$61,LocRow)</f>
-        <v>0</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="C45" s="12">
+        <v>0</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E45" s="2"/>
     </row>
     <row r="46" spans="2:5">
       <c r="B46" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C46" s="12">
+        <v>0</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C46" s="7">
-        <f>INDEX(Locations!$D$2:$D$61,LocRow)</f>
-        <v>0</v>
+      <c r="E46" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="2:5">
       <c r="B47" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="C47" s="7">
-        <f>INDEX(Locations!$E$2:$E$61,LocRow)</f>
-        <v>0</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C48" s="7">
+        <v>74</v>
+      </c>
+      <c r="C48" s="12">
+        <v>0</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="2:5">
+      <c r="B49" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C49" s="14">
+        <v>7.12</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5">
+      <c r="B51" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5">
+      <c r="B52" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="2:5">
+      <c r="B53" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C53" s="14">
+        <v>0.35</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="2:5">
+      <c r="B54" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C54" s="14">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="2:5">
+      <c r="B55" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C55" s="12">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5">
+      <c r="B57" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5">
+      <c r="B58" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C58" s="12">
+        <v>0</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="2:5">
+      <c r="B59" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C59" s="12">
+        <v>0</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="61" spans="2:5">
+      <c r="B61" s="8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5">
+      <c r="B62" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="C62" s="6">
+        <f>MATCH(Location,Locations!$A$2:$A$61,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5">
+      <c r="B63" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C63" s="7">
+        <f>INDEX(Locations!$C$2:$C$61,LocRow)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5">
+      <c r="B64" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C64" s="7">
+        <f>INDEX(Locations!$D$2:$D$61,LocRow)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="2:3">
+      <c r="B65" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C65" s="7">
+        <f>INDEX(Locations!$E$2:$E$61,LocRow)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="2:3">
+      <c r="B66" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C66" s="7">
         <f>INDEX(Locations!$F$2:$F$61,LocRow)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:3">
-      <c r="B49" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C49" s="7">
+    <row r="67" spans="2:3">
+      <c r="B67" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C67" s="7">
         <f>INDEX(Locations!$G$2:$G$61,LocRow)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:3">
-      <c r="B50" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C50" s="7">
-        <f>CornFutures+CornBasis</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="2:3">
-      <c r="B51" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C51" s="7">
-        <f>SbmFutures+SbmBasis</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="2:3">
-      <c r="B52" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C52" s="7">
-        <f>IF(WeanSource="USDA cash (open market)",WeanCash,IF(WeanSource="USDA formula",WeanFormula,WeanManual))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="2:3">
-      <c r="B53" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C53" s="7">
-        <f>HeadPlaced*(1-MortalityPct/100)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="2:3">
-      <c r="B54" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="C54" s="6">
+    <row r="68" spans="2:3">
+      <c r="B68" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C68" s="7">
+        <f>(CornFutures+CornBasis+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="2:3">
+      <c r="B69" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="C69" s="7">
+        <f>(SbmFutures+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="2:3">
+      <c r="B70" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C70" s="7">
+        <f>IF(WeanSource="USDA cash (open market)",WeanCash+WeanAdder,IF(WeanSource="USDA formula",WeanFormula+WeanAdder,WeanManual))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="2:3">
+      <c r="B71" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C71" s="7">
+        <f>IF(MortMode="$ per pig",HeadPlaced,HeadPlaced*(1-MortalityPct/100))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="2:3">
+      <c r="B72" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C72" s="6">
         <f>MAX(Marketing!$A$2:$A$9)+BarnDowntime</f>
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="2:3">
-      <c r="B55" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C55" s="7">
+    <row r="73" spans="2:3">
+      <c r="B73" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C73" s="7">
         <f>HeadSold+(HeadPlaced-HeadSold)*DeadFeedShare</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C17">
       <formula1>"USDA cash (open market),USDA formula,Manual"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C27">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C35">
       <formula1>"$/space/year,$/pig placed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C30">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C38">
       <formula1>"hours x wage,$/pig placed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C12">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9">
+      <formula1>"% of head,$ per pig"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C47">
+      <formula1>"annual rate,$ per pig"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C14">
       <formula1>Locations!$A$2:$A$61</formula1>
     </dataValidation>
   </dataValidations>
@@ -2104,36 +2560,36 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="15" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>85</v>
+      <c r="A2" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>110</v>
       </c>
       <c r="C2" s="12">
         <v>-0.3</v>
@@ -2150,16 +2606,16 @@
       <c r="G2" s="12">
         <v>18.15</v>
       </c>
-      <c r="H2" s="14" t="s">
-        <v>86</v>
+      <c r="H2" s="13" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>88</v>
+      <c r="A3" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>113</v>
       </c>
       <c r="C3" s="12">
         <v>-0.3</v>
@@ -2176,16 +2632,16 @@
       <c r="G3" s="12">
         <v>18.15</v>
       </c>
-      <c r="H3" s="14" t="s">
-        <v>89</v>
+      <c r="H3" s="13" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>91</v>
+      <c r="A4" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="C4" s="12">
         <v>-0.35</v>
@@ -2202,16 +2658,16 @@
       <c r="G4" s="12">
         <v>18.15</v>
       </c>
-      <c r="H4" s="14" t="s">
-        <v>92</v>
+      <c r="H4" s="13" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>94</v>
+      <c r="A5" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>119</v>
       </c>
       <c r="C5" s="12">
         <v>-0.7</v>
@@ -2228,16 +2684,16 @@
       <c r="G5" s="12">
         <v>17.51</v>
       </c>
-      <c r="H5" s="14" t="s">
-        <v>95</v>
+      <c r="H5" s="13" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>94</v>
+      <c r="A6" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>119</v>
       </c>
       <c r="C6" s="12">
         <v>-0.5</v>
@@ -2254,16 +2710,16 @@
       <c r="G6" s="12">
         <v>17.51</v>
       </c>
-      <c r="H6" s="14" t="s">
-        <v>97</v>
+      <c r="H6" s="13" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>91</v>
+      <c r="A7" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="C7" s="12">
         <v>-0.45</v>
@@ -2280,16 +2736,16 @@
       <c r="G7" s="12">
         <v>18.15</v>
       </c>
-      <c r="H7" s="14" t="s">
-        <v>99</v>
+      <c r="H7" s="13" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>101</v>
+      <c r="A8" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>126</v>
       </c>
       <c r="C8" s="12">
         <v>-0.35</v>
@@ -2306,16 +2762,16 @@
       <c r="G8" s="12">
         <v>17.51</v>
       </c>
-      <c r="H8" s="14" t="s">
-        <v>102</v>
+      <c r="H8" s="13" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>104</v>
+      <c r="A9" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>129</v>
       </c>
       <c r="C9" s="12">
         <v>-0.5</v>
@@ -2332,16 +2788,16 @@
       <c r="G9" s="12">
         <v>18.15</v>
       </c>
-      <c r="H9" s="14" t="s">
-        <v>105</v>
+      <c r="H9" s="13" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>91</v>
+      <c r="A10" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="C10" s="12">
         <v>-0.4</v>
@@ -2358,16 +2814,16 @@
       <c r="G10" s="12">
         <v>18.15</v>
       </c>
-      <c r="H10" s="14" t="s">
-        <v>106</v>
+      <c r="H10" s="13" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>108</v>
+      <c r="A11" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>133</v>
       </c>
       <c r="C11" s="12">
         <v>-0.5</v>
@@ -2384,16 +2840,16 @@
       <c r="G11" s="12">
         <v>18.15</v>
       </c>
-      <c r="H11" s="14" t="s">
-        <v>109</v>
+      <c r="H11" s="13" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>91</v>
+      <c r="A12" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="C12" s="12">
         <v>-0.38</v>
@@ -2410,16 +2866,16 @@
       <c r="G12" s="12">
         <v>18.15</v>
       </c>
-      <c r="H12" s="14" t="s">
-        <v>111</v>
+      <c r="H12" s="13" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>108</v>
+      <c r="A13" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>133</v>
       </c>
       <c r="C13" s="12">
         <v>-0.5</v>
@@ -2436,493 +2892,493 @@
       <c r="G13" s="12">
         <v>18.15</v>
       </c>
-      <c r="H13" s="14" t="s">
-        <v>113</v>
+      <c r="H13" s="13" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
       <c r="C14" s="12"/>
       <c r="D14" s="12"/>
       <c r="E14" s="12"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
-      <c r="H14" s="14"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="12"/>
       <c r="D15" s="12"/>
       <c r="E15" s="12"/>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
-      <c r="H15" s="14"/>
+      <c r="H15" s="13"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="12"/>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
-      <c r="H16" s="14"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="12"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
-      <c r="H17" s="14"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="12"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
-      <c r="H18" s="14"/>
+      <c r="H18" s="13"/>
     </row>
     <row r="19" spans="1:8">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="12"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
-      <c r="H19" s="14"/>
+      <c r="H19" s="13"/>
     </row>
     <row r="20" spans="1:8">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="12"/>
       <c r="D20" s="12"/>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
-      <c r="H20" s="14"/>
+      <c r="H20" s="13"/>
     </row>
     <row r="21" spans="1:8">
-      <c r="A21" s="14"/>
-      <c r="B21" s="14"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="12"/>
       <c r="D21" s="12"/>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
-      <c r="H21" s="14"/>
+      <c r="H21" s="13"/>
     </row>
     <row r="22" spans="1:8">
-      <c r="A22" s="14"/>
-      <c r="B22" s="14"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
-      <c r="H22" s="14"/>
+      <c r="H22" s="13"/>
     </row>
     <row r="23" spans="1:8">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
       <c r="C23" s="12"/>
       <c r="D23" s="12"/>
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
-      <c r="H23" s="14"/>
+      <c r="H23" s="13"/>
     </row>
     <row r="24" spans="1:8">
-      <c r="A24" s="14"/>
-      <c r="B24" s="14"/>
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
       <c r="C24" s="12"/>
       <c r="D24" s="12"/>
       <c r="E24" s="12"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="13"/>
     </row>
     <row r="25" spans="1:8">
-      <c r="A25" s="14"/>
-      <c r="B25" s="14"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
-      <c r="H25" s="14"/>
+      <c r="H25" s="13"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="12"/>
       <c r="D26" s="12"/>
       <c r="E26" s="12"/>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
-      <c r="H26" s="14"/>
+      <c r="H26" s="13"/>
     </row>
     <row r="27" spans="1:8">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
       <c r="E27" s="12"/>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
-      <c r="H27" s="14"/>
+      <c r="H27" s="13"/>
     </row>
     <row r="28" spans="1:8">
-      <c r="A28" s="14"/>
-      <c r="B28" s="14"/>
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="12"/>
       <c r="D28" s="12"/>
       <c r="E28" s="12"/>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
-      <c r="H28" s="14"/>
+      <c r="H28" s="13"/>
     </row>
     <row r="29" spans="1:8">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="12"/>
       <c r="D29" s="12"/>
       <c r="E29" s="12"/>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
-      <c r="H29" s="14"/>
+      <c r="H29" s="13"/>
     </row>
     <row r="30" spans="1:8">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="12"/>
       <c r="D30" s="12"/>
       <c r="E30" s="12"/>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
-      <c r="H30" s="14"/>
+      <c r="H30" s="13"/>
     </row>
     <row r="31" spans="1:8">
-      <c r="A31" s="14"/>
-      <c r="B31" s="14"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
       <c r="E31" s="12"/>
       <c r="F31" s="12"/>
       <c r="G31" s="12"/>
-      <c r="H31" s="14"/>
+      <c r="H31" s="13"/>
     </row>
     <row r="32" spans="1:8">
-      <c r="A32" s="14"/>
-      <c r="B32" s="14"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="12"/>
       <c r="D32" s="12"/>
       <c r="E32" s="12"/>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
-      <c r="H32" s="14"/>
+      <c r="H32" s="13"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
-      <c r="H33" s="14"/>
+      <c r="H33" s="13"/>
     </row>
     <row r="34" spans="1:8">
-      <c r="A34" s="14"/>
-      <c r="B34" s="14"/>
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="12"/>
       <c r="D34" s="12"/>
       <c r="E34" s="12"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
-      <c r="H34" s="14"/>
+      <c r="H34" s="13"/>
     </row>
     <row r="35" spans="1:8">
-      <c r="A35" s="14"/>
-      <c r="B35" s="14"/>
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="12"/>
       <c r="D35" s="12"/>
       <c r="E35" s="12"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
-      <c r="H35" s="14"/>
+      <c r="H35" s="13"/>
     </row>
     <row r="36" spans="1:8">
-      <c r="A36" s="14"/>
-      <c r="B36" s="14"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="12"/>
       <c r="D36" s="12"/>
       <c r="E36" s="12"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
-      <c r="H36" s="14"/>
+      <c r="H36" s="13"/>
     </row>
     <row r="37" spans="1:8">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="12"/>
       <c r="D37" s="12"/>
       <c r="E37" s="12"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
-      <c r="H37" s="14"/>
+      <c r="H37" s="13"/>
     </row>
     <row r="38" spans="1:8">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="12"/>
       <c r="D38" s="12"/>
       <c r="E38" s="12"/>
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
-      <c r="H38" s="14"/>
+      <c r="H38" s="13"/>
     </row>
     <row r="39" spans="1:8">
-      <c r="A39" s="14"/>
-      <c r="B39" s="14"/>
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="12"/>
       <c r="D39" s="12"/>
       <c r="E39" s="12"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
-      <c r="H39" s="14"/>
+      <c r="H39" s="13"/>
     </row>
     <row r="40" spans="1:8">
-      <c r="A40" s="14"/>
-      <c r="B40" s="14"/>
+      <c r="A40" s="13"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="12"/>
       <c r="D40" s="12"/>
       <c r="E40" s="12"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
-      <c r="H40" s="14"/>
+      <c r="H40" s="13"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14"/>
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
-      <c r="H41" s="14"/>
+      <c r="H41" s="13"/>
     </row>
     <row r="42" spans="1:8">
-      <c r="A42" s="14"/>
-      <c r="B42" s="14"/>
+      <c r="A42" s="13"/>
+      <c r="B42" s="13"/>
       <c r="C42" s="12"/>
       <c r="D42" s="12"/>
       <c r="E42" s="12"/>
       <c r="F42" s="12"/>
       <c r="G42" s="12"/>
-      <c r="H42" s="14"/>
+      <c r="H42" s="13"/>
     </row>
     <row r="43" spans="1:8">
-      <c r="A43" s="14"/>
-      <c r="B43" s="14"/>
+      <c r="A43" s="13"/>
+      <c r="B43" s="13"/>
       <c r="C43" s="12"/>
       <c r="D43" s="12"/>
       <c r="E43" s="12"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
-      <c r="H43" s="14"/>
+      <c r="H43" s="13"/>
     </row>
     <row r="44" spans="1:8">
-      <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
+      <c r="A44" s="13"/>
+      <c r="B44" s="13"/>
       <c r="C44" s="12"/>
       <c r="D44" s="12"/>
       <c r="E44" s="12"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
-      <c r="H44" s="14"/>
+      <c r="H44" s="13"/>
     </row>
     <row r="45" spans="1:8">
-      <c r="A45" s="14"/>
-      <c r="B45" s="14"/>
+      <c r="A45" s="13"/>
+      <c r="B45" s="13"/>
       <c r="C45" s="12"/>
       <c r="D45" s="12"/>
       <c r="E45" s="12"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
-      <c r="H45" s="14"/>
+      <c r="H45" s="13"/>
     </row>
     <row r="46" spans="1:8">
-      <c r="A46" s="14"/>
-      <c r="B46" s="14"/>
+      <c r="A46" s="13"/>
+      <c r="B46" s="13"/>
       <c r="C46" s="12"/>
       <c r="D46" s="12"/>
       <c r="E46" s="12"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
-      <c r="H46" s="14"/>
+      <c r="H46" s="13"/>
     </row>
     <row r="47" spans="1:8">
-      <c r="A47" s="14"/>
-      <c r="B47" s="14"/>
+      <c r="A47" s="13"/>
+      <c r="B47" s="13"/>
       <c r="C47" s="12"/>
       <c r="D47" s="12"/>
       <c r="E47" s="12"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
-      <c r="H47" s="14"/>
+      <c r="H47" s="13"/>
     </row>
     <row r="48" spans="1:8">
-      <c r="A48" s="14"/>
-      <c r="B48" s="14"/>
+      <c r="A48" s="13"/>
+      <c r="B48" s="13"/>
       <c r="C48" s="12"/>
       <c r="D48" s="12"/>
       <c r="E48" s="12"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
-      <c r="H48" s="14"/>
+      <c r="H48" s="13"/>
     </row>
     <row r="49" spans="1:8">
-      <c r="A49" s="14"/>
-      <c r="B49" s="14"/>
+      <c r="A49" s="13"/>
+      <c r="B49" s="13"/>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
       <c r="E49" s="12"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
-      <c r="H49" s="14"/>
+      <c r="H49" s="13"/>
     </row>
     <row r="50" spans="1:8">
-      <c r="A50" s="14"/>
-      <c r="B50" s="14"/>
+      <c r="A50" s="13"/>
+      <c r="B50" s="13"/>
       <c r="C50" s="12"/>
       <c r="D50" s="12"/>
       <c r="E50" s="12"/>
       <c r="F50" s="12"/>
       <c r="G50" s="12"/>
-      <c r="H50" s="14"/>
+      <c r="H50" s="13"/>
     </row>
     <row r="51" spans="1:8">
-      <c r="A51" s="14"/>
-      <c r="B51" s="14"/>
+      <c r="A51" s="13"/>
+      <c r="B51" s="13"/>
       <c r="C51" s="12"/>
       <c r="D51" s="12"/>
       <c r="E51" s="12"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
-      <c r="H51" s="14"/>
+      <c r="H51" s="13"/>
     </row>
     <row r="52" spans="1:8">
-      <c r="A52" s="14"/>
-      <c r="B52" s="14"/>
+      <c r="A52" s="13"/>
+      <c r="B52" s="13"/>
       <c r="C52" s="12"/>
       <c r="D52" s="12"/>
       <c r="E52" s="12"/>
       <c r="F52" s="12"/>
       <c r="G52" s="12"/>
-      <c r="H52" s="14"/>
+      <c r="H52" s="13"/>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="14"/>
-      <c r="B53" s="14"/>
+      <c r="A53" s="13"/>
+      <c r="B53" s="13"/>
       <c r="C53" s="12"/>
       <c r="D53" s="12"/>
       <c r="E53" s="12"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
-      <c r="H53" s="14"/>
+      <c r="H53" s="13"/>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="14"/>
-      <c r="B54" s="14"/>
+      <c r="A54" s="13"/>
+      <c r="B54" s="13"/>
       <c r="C54" s="12"/>
       <c r="D54" s="12"/>
       <c r="E54" s="12"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
-      <c r="H54" s="14"/>
+      <c r="H54" s="13"/>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="14"/>
-      <c r="B55" s="14"/>
+      <c r="A55" s="13"/>
+      <c r="B55" s="13"/>
       <c r="C55" s="12"/>
       <c r="D55" s="12"/>
       <c r="E55" s="12"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
-      <c r="H55" s="14"/>
+      <c r="H55" s="13"/>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" s="14"/>
-      <c r="B56" s="14"/>
+      <c r="A56" s="13"/>
+      <c r="B56" s="13"/>
       <c r="C56" s="12"/>
       <c r="D56" s="12"/>
       <c r="E56" s="12"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
-      <c r="H56" s="14"/>
+      <c r="H56" s="13"/>
     </row>
     <row r="57" spans="1:8">
-      <c r="A57" s="14"/>
-      <c r="B57" s="14"/>
+      <c r="A57" s="13"/>
+      <c r="B57" s="13"/>
       <c r="C57" s="12"/>
       <c r="D57" s="12"/>
       <c r="E57" s="12"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
-      <c r="H57" s="14"/>
+      <c r="H57" s="13"/>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="14"/>
-      <c r="B58" s="14"/>
+      <c r="A58" s="13"/>
+      <c r="B58" s="13"/>
       <c r="C58" s="12"/>
       <c r="D58" s="12"/>
       <c r="E58" s="12"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
-      <c r="H58" s="14"/>
+      <c r="H58" s="13"/>
     </row>
     <row r="59" spans="1:8">
-      <c r="A59" s="14"/>
-      <c r="B59" s="14"/>
+      <c r="A59" s="13"/>
+      <c r="B59" s="13"/>
       <c r="C59" s="12"/>
       <c r="D59" s="12"/>
       <c r="E59" s="12"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
-      <c r="H59" s="14"/>
+      <c r="H59" s="13"/>
     </row>
     <row r="60" spans="1:8">
-      <c r="A60" s="14"/>
-      <c r="B60" s="14"/>
+      <c r="A60" s="13"/>
+      <c r="B60" s="13"/>
       <c r="C60" s="12"/>
       <c r="D60" s="12"/>
       <c r="E60" s="12"/>
       <c r="F60" s="12"/>
       <c r="G60" s="12"/>
-      <c r="H60" s="14"/>
+      <c r="H60" s="13"/>
     </row>
     <row r="61" spans="1:8">
-      <c r="A61" s="14"/>
-      <c r="B61" s="14"/>
+      <c r="A61" s="13"/>
+      <c r="B61" s="13"/>
       <c r="C61" s="12"/>
       <c r="D61" s="12"/>
       <c r="E61" s="12"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
-      <c r="H61" s="14"/>
+      <c r="H61" s="13"/>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" s="2" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2945,51 +3401,51 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="15" t="s">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>119</v>
+        <v>144</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="14" t="s">
-        <v>128</v>
+      <c r="A2" s="13" t="s">
+        <v>153</v>
       </c>
       <c r="B2" s="12">
         <v>20</v>
@@ -3040,8 +3496,8 @@
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" s="14" t="s">
-        <v>129</v>
+      <c r="A3" s="13" t="s">
+        <v>154</v>
       </c>
       <c r="B3" s="12">
         <v>35</v>
@@ -3092,8 +3548,8 @@
       </c>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" s="14" t="s">
-        <v>130</v>
+      <c r="A4" s="13" t="s">
+        <v>155</v>
       </c>
       <c r="B4" s="12">
         <v>120</v>
@@ -3144,8 +3600,8 @@
       </c>
     </row>
     <row r="5" spans="1:14">
-      <c r="A5" s="14" t="s">
-        <v>131</v>
+      <c r="A5" s="13" t="s">
+        <v>156</v>
       </c>
       <c r="B5" s="12">
         <v>160</v>
@@ -3196,8 +3652,8 @@
       </c>
     </row>
     <row r="6" spans="1:14">
-      <c r="A6" s="14" t="s">
-        <v>132</v>
+      <c r="A6" s="13" t="s">
+        <v>157</v>
       </c>
       <c r="B6" s="12">
         <v>180</v>
@@ -3248,8 +3704,8 @@
       </c>
     </row>
     <row r="7" spans="1:14">
-      <c r="A7" s="14" t="s">
-        <v>133</v>
+      <c r="A7" s="13" t="s">
+        <v>158</v>
       </c>
       <c r="B7" s="12">
         <v>195</v>
@@ -3300,7 +3756,7 @@
       </c>
     </row>
     <row r="8" spans="1:14">
-      <c r="A8" s="14"/>
+      <c r="A8" s="13"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
       <c r="D8" s="12"/>
@@ -3340,7 +3796,7 @@
       </c>
     </row>
     <row r="9" spans="1:14">
-      <c r="A9" s="14"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
       <c r="D9" s="12"/>
@@ -3380,7 +3836,7 @@
       </c>
     </row>
     <row r="10" spans="1:14">
-      <c r="A10" s="14"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -3420,7 +3876,7 @@
       </c>
     </row>
     <row r="11" spans="1:14">
-      <c r="A11" s="14"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -3460,7 +3916,7 @@
       </c>
     </row>
     <row r="12" spans="1:14">
-      <c r="A12" s="14"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -3500,7 +3956,7 @@
       </c>
     </row>
     <row r="13" spans="1:14">
-      <c r="A13" s="14"/>
+      <c r="A13" s="13"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -3541,7 +3997,7 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="8" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="B14" s="7">
         <f>SUM(B2:B13)</f>
@@ -3578,7 +4034,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="2" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -3600,50 +4056,50 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="15" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>169</v>
+        <v>194</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>170</v>
+        <v>195</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>177</v>
+        <v>202</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="10">
         <v>145</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="14">
         <v>20</v>
       </c>
       <c r="C2" s="12">
@@ -3662,7 +4118,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="7">
-        <f>IF(AND(A2&lt;&gt;"",N(B2)&gt;0),INDEX(FutPrices,MATCH(E2,FutContracts,0)),0)</f>
+        <f>IF(AND(A2&lt;&gt;"",N(B2)&gt;0),INDEX(FutPrices,MATCH(E2,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H2" s="7">
@@ -3694,7 +4150,7 @@
       <c r="A3" s="10">
         <v>160</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="14">
         <v>40</v>
       </c>
       <c r="C3" s="12">
@@ -3713,7 +4169,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="7">
-        <f>IF(AND(A3&lt;&gt;"",N(B3)&gt;0),INDEX(FutPrices,MATCH(E3,FutContracts,0)),0)</f>
+        <f>IF(AND(A3&lt;&gt;"",N(B3)&gt;0),INDEX(FutPrices,MATCH(E3,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H3" s="7">
@@ -3745,7 +4201,7 @@
       <c r="A4" s="10">
         <v>175</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="14">
         <v>40</v>
       </c>
       <c r="C4" s="12">
@@ -3764,7 +4220,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="7">
-        <f>IF(AND(A4&lt;&gt;"",N(B4)&gt;0),INDEX(FutPrices,MATCH(E4,FutContracts,0)),0)</f>
+        <f>IF(AND(A4&lt;&gt;"",N(B4)&gt;0),INDEX(FutPrices,MATCH(E4,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H4" s="7">
@@ -3809,7 +4265,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="7">
-        <f>IF(AND(A5&lt;&gt;"",N(B5)&gt;0),INDEX(FutPrices,MATCH(E5,FutContracts,0)),0)</f>
+        <f>IF(AND(A5&lt;&gt;"",N(B5)&gt;0),INDEX(FutPrices,MATCH(E5,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="7">
@@ -3854,7 +4310,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="7">
-        <f>IF(AND(A6&lt;&gt;"",N(B6)&gt;0),INDEX(FutPrices,MATCH(E6,FutContracts,0)),0)</f>
+        <f>IF(AND(A6&lt;&gt;"",N(B6)&gt;0),INDEX(FutPrices,MATCH(E6,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H6" s="7">
@@ -3899,7 +4355,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="7">
-        <f>IF(AND(A7&lt;&gt;"",N(B7)&gt;0),INDEX(FutPrices,MATCH(E7,FutContracts,0)),0)</f>
+        <f>IF(AND(A7&lt;&gt;"",N(B7)&gt;0),INDEX(FutPrices,MATCH(E7,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H7" s="7">
@@ -3944,7 +4400,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="7">
-        <f>IF(AND(A8&lt;&gt;"",N(B8)&gt;0),INDEX(FutPrices,MATCH(E8,FutContracts,0)),0)</f>
+        <f>IF(AND(A8&lt;&gt;"",N(B8)&gt;0),INDEX(FutPrices,MATCH(E8,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H8" s="7">
@@ -3989,7 +4445,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="7">
-        <f>IF(AND(A9&lt;&gt;"",N(B9)&gt;0),INDEX(FutPrices,MATCH(E9,FutContracts,0)),0)</f>
+        <f>IF(AND(A9&lt;&gt;"",N(B9)&gt;0),INDEX(FutPrices,MATCH(E9,FutContracts,0))*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100,0)</f>
         <v>0</v>
       </c>
       <c r="H9" s="7">
@@ -4019,7 +4475,7 @@
     </row>
     <row r="10" spans="1:13">
       <c r="A10" s="8" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="B10" s="7">
         <f>SUM(B2:B9)</f>
@@ -4036,7 +4492,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="2" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -4067,32 +4523,32 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="8" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>141</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="15" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>142</v>
+        <v>167</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>143</v>
+        <v>168</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="14" t="s">
-        <v>138</v>
+      <c r="A3" s="13" t="s">
+        <v>163</v>
       </c>
       <c r="B3" s="12">
         <v>66.925</v>
@@ -4101,15 +4557,15 @@
         <v>1</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="F3" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="14" t="s">
-        <v>139</v>
+      <c r="A4" s="13" t="s">
+        <v>164</v>
       </c>
       <c r="B4" s="12">
         <v>69.22499999999999</v>
@@ -4118,15 +4574,15 @@
         <v>2</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="F4" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="14" t="s">
-        <v>140</v>
+      <c r="A5" s="13" t="s">
+        <v>165</v>
       </c>
       <c r="B5" s="12">
         <v>74.675</v>
@@ -4135,280 +4591,280 @@
         <v>3</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
       <c r="F5" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="14"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="12"/>
       <c r="D6" s="6">
         <v>4</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>147</v>
+        <v>172</v>
       </c>
       <c r="F6" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="14"/>
+      <c r="A7" s="13"/>
       <c r="B7" s="12"/>
       <c r="D7" s="6">
         <v>5</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="F7" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="14"/>
+      <c r="A8" s="13"/>
       <c r="B8" s="12"/>
       <c r="D8" s="6">
         <v>6</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="F8" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="14"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="12"/>
       <c r="D9" s="6">
         <v>7</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="F9" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="14"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="12"/>
       <c r="D10" s="6">
         <v>8</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="F10" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="14"/>
+      <c r="A11" s="13"/>
       <c r="B11" s="12"/>
       <c r="D11" s="6">
         <v>9</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>152</v>
+        <v>177</v>
       </c>
       <c r="F11" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="14"/>
+      <c r="A12" s="13"/>
       <c r="B12" s="12"/>
       <c r="D12" s="6">
         <v>10</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>153</v>
+        <v>178</v>
       </c>
       <c r="F12" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="14"/>
+      <c r="A13" s="13"/>
       <c r="B13" s="12"/>
       <c r="D13" s="6">
         <v>11</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="F13" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="14"/>
+      <c r="A14" s="13"/>
       <c r="B14" s="12"/>
       <c r="D14" s="6">
         <v>12</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="F14" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="14"/>
+      <c r="A15" s="13"/>
       <c r="B15" s="12"/>
       <c r="D15" s="6">
         <v>13</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>156</v>
+        <v>181</v>
       </c>
       <c r="F15" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="14"/>
+      <c r="A16" s="13"/>
       <c r="B16" s="12"/>
       <c r="D16" s="6">
         <v>14</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>157</v>
+        <v>182</v>
       </c>
       <c r="F16" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="14"/>
+      <c r="A17" s="13"/>
       <c r="B17" s="12"/>
       <c r="D17" s="6">
         <v>15</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>158</v>
+        <v>183</v>
       </c>
       <c r="F17" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="14"/>
+      <c r="A18" s="13"/>
       <c r="B18" s="12"/>
       <c r="D18" s="6">
         <v>16</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="F18" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="14"/>
+      <c r="A19" s="13"/>
       <c r="B19" s="12"/>
       <c r="D19" s="6">
         <v>17</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="F19" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="14"/>
+      <c r="A20" s="13"/>
       <c r="B20" s="12"/>
       <c r="D20" s="6">
         <v>18</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="F20" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="14"/>
+      <c r="A21" s="13"/>
       <c r="B21" s="12"/>
       <c r="D21" s="6">
         <v>19</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="F21" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="14"/>
+      <c r="A22" s="13"/>
       <c r="B22" s="12"/>
       <c r="D22" s="6">
         <v>20</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
       <c r="F22" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="14"/>
+      <c r="A23" s="13"/>
       <c r="B23" s="12"/>
       <c r="D23" s="6">
         <v>21</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="F23" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="14"/>
+      <c r="A24" s="13"/>
       <c r="B24" s="12"/>
       <c r="D24" s="6">
         <v>22</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="F24" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="14"/>
+      <c r="A25" s="13"/>
       <c r="B25" s="12"/>
       <c r="D25" s="6">
         <v>23</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="F25" s="12">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="14"/>
+      <c r="A26" s="13"/>
       <c r="B26" s="12"/>
       <c r="D26" s="6">
         <v>24</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
       <c r="F26" s="12">
         <v>0</v>
@@ -4425,7 +4881,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -4434,27 +4890,27 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="15" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="9" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="B2" s="4">
         <f>HeadPlaced*(WeanPrice+WeanFreight)</f>
@@ -4473,13 +4929,13 @@
         <v>0</v>
       </c>
       <c r="F2" s="18">
-        <f>B2/$B$12</f>
+        <f>B2/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="9" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
       <c r="B3" s="4">
         <f>FeedCost</f>
@@ -4498,13 +4954,13 @@
         <v>0</v>
       </c>
       <c r="F3" s="18">
-        <f>B3/$B$12</f>
+        <f>B3/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>186</v>
+        <v>211</v>
       </c>
       <c r="B4" s="4">
         <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*BarnDays/365,HeadPlaced*BarnPerPig)</f>
@@ -4523,13 +4979,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="18">
-        <f>B4/$B$12</f>
+        <f>B4/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="9" t="s">
-        <v>187</v>
+        <v>212</v>
       </c>
       <c r="B5" s="4">
         <f>IF(LaborMode="hours x wage",HeadPlaced*LaborHours*LaborWage,HeadPlaced*LaborPerPig)</f>
@@ -4548,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="F5" s="18">
-        <f>B5/$B$12</f>
+        <f>B5/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="B6" s="4">
         <f>HeadPlaced*VetMed</f>
@@ -4573,13 +5029,13 @@
         <v>0</v>
       </c>
       <c r="F6" s="18">
-        <f>B6/$B$12</f>
+        <f>B6/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>189</v>
+        <v>214</v>
       </c>
       <c r="B7" s="4">
         <f>HeadPlaced*Utilities</f>
@@ -4598,13 +5054,13 @@
         <v>0</v>
       </c>
       <c r="F7" s="18">
-        <f>B7/$B$12</f>
+        <f>B7/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="9" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B8" s="4">
         <f>HeadSold*Trucking</f>
@@ -4623,13 +5079,13 @@
         <v>0</v>
       </c>
       <c r="F8" s="18">
-        <f>B8/$B$12</f>
+        <f>B8/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="9" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B9" s="4">
         <f>HeadPlaced*InsMisc</f>
@@ -4648,16 +5104,16 @@
         <v>0</v>
       </c>
       <c r="F9" s="18">
-        <f>B9/$B$12</f>
+        <f>B9/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>190</v>
+        <v>69</v>
       </c>
       <c r="B10" s="4">
-        <f>InterestPct/100*AvgDays/365*(B2+0.5*B3)</f>
+        <f>HeadPlaced*GA</f>
         <v>0</v>
       </c>
       <c r="C10" s="5">
@@ -4673,16 +5129,16 @@
         <v>0</v>
       </c>
       <c r="F10" s="18">
-        <f>B10/$B$12</f>
+        <f>B10/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>191</v>
+        <v>215</v>
       </c>
       <c r="B11" s="4">
-        <f>GrossRevenue*CheckoffPct/100</f>
+        <f>IF(MortMode="$ per pig",HeadPlaced*MortCost,0)</f>
         <v>0</v>
       </c>
       <c r="C11" s="5">
@@ -4698,28 +5154,103 @@
         <v>0</v>
       </c>
       <c r="F11" s="18">
-        <f>B11/$B$12</f>
+        <f>B11/$B$15</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="B12" s="16">
-        <f>SUM(B2:B11)</f>
-        <v>0</v>
-      </c>
-      <c r="C12" s="19">
+      <c r="A12" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B12" s="4">
+        <f>HeadSold*OtherSold</f>
+        <v>0</v>
+      </c>
+      <c r="C12" s="5">
         <f>B12/HeadPlaced</f>
         <v>0</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="5">
         <f>B12/HeadSold</f>
         <v>0</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="5">
         <f>B12/CarcassCwt</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="18">
+        <f>B12/$B$15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B13" s="4">
+        <f>IF(InterestMode="annual rate",InterestPct/100*AvgDays/365*(B2+0.5*B3),HeadPlaced*InterestPerPig)</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="5">
+        <f>B13/HeadPlaced</f>
+        <v>0</v>
+      </c>
+      <c r="D13" s="5">
+        <f>B13/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
+        <f>B13/CarcassCwt</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="18">
+        <f>B13/$B$15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="4">
+        <f>GrossRevenue*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="5">
+        <f>B14/HeadPlaced</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="5">
+        <f>B14/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
+        <f>B14/CarcassCwt</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="18">
+        <f>B14/$B$15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="16">
+        <f>SUM(B2:B14)</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="19">
+        <f>B15/HeadPlaced</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="19">
+        <f>B15/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="19">
+        <f>B15/CarcassCwt</f>
         <v>0</v>
       </c>
     </row>
@@ -4727,4 +5258,1204 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M32"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
+    <col min="2" max="14" width="13.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="2" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B5" s="10">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="B6" s="12">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="B9" s="11">
+        <v>46313</v>
+      </c>
+      <c r="C9" s="11">
+        <v>46306</v>
+      </c>
+      <c r="D9" s="11">
+        <v>46299</v>
+      </c>
+      <c r="E9" s="11">
+        <v>46292</v>
+      </c>
+      <c r="F9" s="11">
+        <v>46285</v>
+      </c>
+      <c r="G9" s="11">
+        <v>46278</v>
+      </c>
+      <c r="H9" s="11">
+        <v>46271</v>
+      </c>
+      <c r="I9" s="11">
+        <v>46264</v>
+      </c>
+      <c r="J9" s="11">
+        <v>46257</v>
+      </c>
+      <c r="K9" s="11">
+        <v>46250</v>
+      </c>
+      <c r="L9" s="11">
+        <v>46243</v>
+      </c>
+      <c r="M9" s="11">
+        <v>46236</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
+      <c r="A10" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="B10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="C10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="D10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="E10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="F10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="G10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="H10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="I10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="J10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="K10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="L10" s="12">
+        <v>24.81</v>
+      </c>
+      <c r="M10" s="12">
+        <v>24.81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="C11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="D11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="E11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="F11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="G11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="H11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="I11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="J11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="K11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="L11" s="12">
+        <v>4.7425</v>
+      </c>
+      <c r="M11" s="12">
+        <v>4.7425</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="B12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="C12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="D12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="E12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="F12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="G12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="H12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="I12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="J12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="K12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="L12" s="12">
+        <v>357.1</v>
+      </c>
+      <c r="M12" s="12">
+        <v>357.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" s="12">
+        <v>180</v>
+      </c>
+      <c r="C13" s="12">
+        <v>180</v>
+      </c>
+      <c r="D13" s="12">
+        <v>180</v>
+      </c>
+      <c r="E13" s="12">
+        <v>180</v>
+      </c>
+      <c r="F13" s="12">
+        <v>180</v>
+      </c>
+      <c r="G13" s="12">
+        <v>180</v>
+      </c>
+      <c r="H13" s="12">
+        <v>180</v>
+      </c>
+      <c r="I13" s="12">
+        <v>180</v>
+      </c>
+      <c r="J13" s="12">
+        <v>180</v>
+      </c>
+      <c r="K13" s="12">
+        <v>180</v>
+      </c>
+      <c r="L13" s="12">
+        <v>180</v>
+      </c>
+      <c r="M13" s="12">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B14" s="12">
+        <v>74.675</v>
+      </c>
+      <c r="C14" s="12">
+        <v>74.675</v>
+      </c>
+      <c r="D14" s="12">
+        <v>74.675</v>
+      </c>
+      <c r="E14" s="12">
+        <v>74.675</v>
+      </c>
+      <c r="F14" s="12">
+        <v>74.675</v>
+      </c>
+      <c r="G14" s="12">
+        <v>74.675</v>
+      </c>
+      <c r="H14" s="12">
+        <v>69.22499999999999</v>
+      </c>
+      <c r="I14" s="12">
+        <v>69.22499999999999</v>
+      </c>
+      <c r="J14" s="12">
+        <v>69.22499999999999</v>
+      </c>
+      <c r="K14" s="12">
+        <v>69.22499999999999</v>
+      </c>
+      <c r="L14" s="12">
+        <v>69.22499999999999</v>
+      </c>
+      <c r="M14" s="12">
+        <v>69.22499999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="B15" s="12">
+        <v>0</v>
+      </c>
+      <c r="C15" s="12">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12">
+        <v>0</v>
+      </c>
+      <c r="E15" s="12">
+        <v>0</v>
+      </c>
+      <c r="F15" s="12">
+        <v>0</v>
+      </c>
+      <c r="G15" s="12">
+        <v>0</v>
+      </c>
+      <c r="H15" s="12">
+        <v>0</v>
+      </c>
+      <c r="I15" s="12">
+        <v>0</v>
+      </c>
+      <c r="J15" s="12">
+        <v>0</v>
+      </c>
+      <c r="K15" s="12">
+        <v>0</v>
+      </c>
+      <c r="L15" s="12">
+        <v>0</v>
+      </c>
+      <c r="M15" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="17">
+        <f>B9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="17">
+        <f>C9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="D17" s="17">
+        <f>D9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="17">
+        <f>E9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="17">
+        <f>F9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="17">
+        <f>G9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="H17" s="17">
+        <f>H9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="17">
+        <f>I9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="17">
+        <f>J9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="K17" s="17">
+        <f>K9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="L17" s="17">
+        <f>L9+CrLag</f>
+        <v>0</v>
+      </c>
+      <c r="M17" s="17">
+        <f>M9+CrLag</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B18" s="17">
+        <f>B17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="17">
+        <f>C17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="17">
+        <f>D17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="17">
+        <f>E17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="F18" s="17">
+        <f>F17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="17">
+        <f>G17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="17">
+        <f>H17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="17">
+        <f>I17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="17">
+        <f>J17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="K18" s="17">
+        <f>K17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="L18" s="17">
+        <f>L17+CrDays</f>
+        <v>0</v>
+      </c>
+      <c r="M18" s="17">
+        <f>M17+CrDays</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" s="20">
+        <f>(YEAR(B18)+(IF(AND(ISNUMBER(MATCH(MONTH(B18),{2,4,5,6,7,8,10,12},0)),DAY(B18)&lt;=14),MONTH(B18),IF(MONTH(B18)&lt;2,2,IF(MONTH(B18)&lt;4,4,IF(MONTH(B18)&lt;8,MONTH(B18)+1,IF(MONTH(B18)&lt;10,10,IF(MONTH(B18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(B18),{2,4,5,6,7,8,10,12},0)),DAY(B18)&lt;=14),MONTH(B18),IF(MONTH(B18)&lt;2,2,IF(MONTH(B18)&lt;4,4,IF(MONTH(B18)&lt;8,MONTH(B18)+1,IF(MONTH(B18)&lt;10,10,IF(MONTH(B18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(B18),{2,4,5,6,7,8,10,12},0)),DAY(B18)&lt;=14),MONTH(B18),IF(MONTH(B18)&lt;2,2,IF(MONTH(B18)&lt;4,4,IF(MONTH(B18)&lt;8,MONTH(B18)+1,IF(MONTH(B18)&lt;10,10,IF(MONTH(B18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="20">
+        <f>(YEAR(C18)+(IF(AND(ISNUMBER(MATCH(MONTH(C18),{2,4,5,6,7,8,10,12},0)),DAY(C18)&lt;=14),MONTH(C18),IF(MONTH(C18)&lt;2,2,IF(MONTH(C18)&lt;4,4,IF(MONTH(C18)&lt;8,MONTH(C18)+1,IF(MONTH(C18)&lt;10,10,IF(MONTH(C18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(C18),{2,4,5,6,7,8,10,12},0)),DAY(C18)&lt;=14),MONTH(C18),IF(MONTH(C18)&lt;2,2,IF(MONTH(C18)&lt;4,4,IF(MONTH(C18)&lt;8,MONTH(C18)+1,IF(MONTH(C18)&lt;10,10,IF(MONTH(C18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(C18),{2,4,5,6,7,8,10,12},0)),DAY(C18)&lt;=14),MONTH(C18),IF(MONTH(C18)&lt;2,2,IF(MONTH(C18)&lt;4,4,IF(MONTH(C18)&lt;8,MONTH(C18)+1,IF(MONTH(C18)&lt;10,10,IF(MONTH(C18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="20">
+        <f>(YEAR(D18)+(IF(AND(ISNUMBER(MATCH(MONTH(D18),{2,4,5,6,7,8,10,12},0)),DAY(D18)&lt;=14),MONTH(D18),IF(MONTH(D18)&lt;2,2,IF(MONTH(D18)&lt;4,4,IF(MONTH(D18)&lt;8,MONTH(D18)+1,IF(MONTH(D18)&lt;10,10,IF(MONTH(D18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(D18),{2,4,5,6,7,8,10,12},0)),DAY(D18)&lt;=14),MONTH(D18),IF(MONTH(D18)&lt;2,2,IF(MONTH(D18)&lt;4,4,IF(MONTH(D18)&lt;8,MONTH(D18)+1,IF(MONTH(D18)&lt;10,10,IF(MONTH(D18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(D18),{2,4,5,6,7,8,10,12},0)),DAY(D18)&lt;=14),MONTH(D18),IF(MONTH(D18)&lt;2,2,IF(MONTH(D18)&lt;4,4,IF(MONTH(D18)&lt;8,MONTH(D18)+1,IF(MONTH(D18)&lt;10,10,IF(MONTH(D18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="20">
+        <f>(YEAR(E18)+(IF(AND(ISNUMBER(MATCH(MONTH(E18),{2,4,5,6,7,8,10,12},0)),DAY(E18)&lt;=14),MONTH(E18),IF(MONTH(E18)&lt;2,2,IF(MONTH(E18)&lt;4,4,IF(MONTH(E18)&lt;8,MONTH(E18)+1,IF(MONTH(E18)&lt;10,10,IF(MONTH(E18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(E18),{2,4,5,6,7,8,10,12},0)),DAY(E18)&lt;=14),MONTH(E18),IF(MONTH(E18)&lt;2,2,IF(MONTH(E18)&lt;4,4,IF(MONTH(E18)&lt;8,MONTH(E18)+1,IF(MONTH(E18)&lt;10,10,IF(MONTH(E18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(E18),{2,4,5,6,7,8,10,12},0)),DAY(E18)&lt;=14),MONTH(E18),IF(MONTH(E18)&lt;2,2,IF(MONTH(E18)&lt;4,4,IF(MONTH(E18)&lt;8,MONTH(E18)+1,IF(MONTH(E18)&lt;10,10,IF(MONTH(E18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="20">
+        <f>(YEAR(F18)+(IF(AND(ISNUMBER(MATCH(MONTH(F18),{2,4,5,6,7,8,10,12},0)),DAY(F18)&lt;=14),MONTH(F18),IF(MONTH(F18)&lt;2,2,IF(MONTH(F18)&lt;4,4,IF(MONTH(F18)&lt;8,MONTH(F18)+1,IF(MONTH(F18)&lt;10,10,IF(MONTH(F18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(F18),{2,4,5,6,7,8,10,12},0)),DAY(F18)&lt;=14),MONTH(F18),IF(MONTH(F18)&lt;2,2,IF(MONTH(F18)&lt;4,4,IF(MONTH(F18)&lt;8,MONTH(F18)+1,IF(MONTH(F18)&lt;10,10,IF(MONTH(F18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(F18),{2,4,5,6,7,8,10,12},0)),DAY(F18)&lt;=14),MONTH(F18),IF(MONTH(F18)&lt;2,2,IF(MONTH(F18)&lt;4,4,IF(MONTH(F18)&lt;8,MONTH(F18)+1,IF(MONTH(F18)&lt;10,10,IF(MONTH(F18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="20">
+        <f>(YEAR(G18)+(IF(AND(ISNUMBER(MATCH(MONTH(G18),{2,4,5,6,7,8,10,12},0)),DAY(G18)&lt;=14),MONTH(G18),IF(MONTH(G18)&lt;2,2,IF(MONTH(G18)&lt;4,4,IF(MONTH(G18)&lt;8,MONTH(G18)+1,IF(MONTH(G18)&lt;10,10,IF(MONTH(G18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(G18),{2,4,5,6,7,8,10,12},0)),DAY(G18)&lt;=14),MONTH(G18),IF(MONTH(G18)&lt;2,2,IF(MONTH(G18)&lt;4,4,IF(MONTH(G18)&lt;8,MONTH(G18)+1,IF(MONTH(G18)&lt;10,10,IF(MONTH(G18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(G18),{2,4,5,6,7,8,10,12},0)),DAY(G18)&lt;=14),MONTH(G18),IF(MONTH(G18)&lt;2,2,IF(MONTH(G18)&lt;4,4,IF(MONTH(G18)&lt;8,MONTH(G18)+1,IF(MONTH(G18)&lt;10,10,IF(MONTH(G18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="20">
+        <f>(YEAR(H18)+(IF(AND(ISNUMBER(MATCH(MONTH(H18),{2,4,5,6,7,8,10,12},0)),DAY(H18)&lt;=14),MONTH(H18),IF(MONTH(H18)&lt;2,2,IF(MONTH(H18)&lt;4,4,IF(MONTH(H18)&lt;8,MONTH(H18)+1,IF(MONTH(H18)&lt;10,10,IF(MONTH(H18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(H18),{2,4,5,6,7,8,10,12},0)),DAY(H18)&lt;=14),MONTH(H18),IF(MONTH(H18)&lt;2,2,IF(MONTH(H18)&lt;4,4,IF(MONTH(H18)&lt;8,MONTH(H18)+1,IF(MONTH(H18)&lt;10,10,IF(MONTH(H18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(H18),{2,4,5,6,7,8,10,12},0)),DAY(H18)&lt;=14),MONTH(H18),IF(MONTH(H18)&lt;2,2,IF(MONTH(H18)&lt;4,4,IF(MONTH(H18)&lt;8,MONTH(H18)+1,IF(MONTH(H18)&lt;10,10,IF(MONTH(H18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="20">
+        <f>(YEAR(I18)+(IF(AND(ISNUMBER(MATCH(MONTH(I18),{2,4,5,6,7,8,10,12},0)),DAY(I18)&lt;=14),MONTH(I18),IF(MONTH(I18)&lt;2,2,IF(MONTH(I18)&lt;4,4,IF(MONTH(I18)&lt;8,MONTH(I18)+1,IF(MONTH(I18)&lt;10,10,IF(MONTH(I18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(I18),{2,4,5,6,7,8,10,12},0)),DAY(I18)&lt;=14),MONTH(I18),IF(MONTH(I18)&lt;2,2,IF(MONTH(I18)&lt;4,4,IF(MONTH(I18)&lt;8,MONTH(I18)+1,IF(MONTH(I18)&lt;10,10,IF(MONTH(I18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(I18),{2,4,5,6,7,8,10,12},0)),DAY(I18)&lt;=14),MONTH(I18),IF(MONTH(I18)&lt;2,2,IF(MONTH(I18)&lt;4,4,IF(MONTH(I18)&lt;8,MONTH(I18)+1,IF(MONTH(I18)&lt;10,10,IF(MONTH(I18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="20">
+        <f>(YEAR(J18)+(IF(AND(ISNUMBER(MATCH(MONTH(J18),{2,4,5,6,7,8,10,12},0)),DAY(J18)&lt;=14),MONTH(J18),IF(MONTH(J18)&lt;2,2,IF(MONTH(J18)&lt;4,4,IF(MONTH(J18)&lt;8,MONTH(J18)+1,IF(MONTH(J18)&lt;10,10,IF(MONTH(J18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(J18),{2,4,5,6,7,8,10,12},0)),DAY(J18)&lt;=14),MONTH(J18),IF(MONTH(J18)&lt;2,2,IF(MONTH(J18)&lt;4,4,IF(MONTH(J18)&lt;8,MONTH(J18)+1,IF(MONTH(J18)&lt;10,10,IF(MONTH(J18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(J18),{2,4,5,6,7,8,10,12},0)),DAY(J18)&lt;=14),MONTH(J18),IF(MONTH(J18)&lt;2,2,IF(MONTH(J18)&lt;4,4,IF(MONTH(J18)&lt;8,MONTH(J18)+1,IF(MONTH(J18)&lt;10,10,IF(MONTH(J18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="K19" s="20">
+        <f>(YEAR(K18)+(IF(AND(ISNUMBER(MATCH(MONTH(K18),{2,4,5,6,7,8,10,12},0)),DAY(K18)&lt;=14),MONTH(K18),IF(MONTH(K18)&lt;2,2,IF(MONTH(K18)&lt;4,4,IF(MONTH(K18)&lt;8,MONTH(K18)+1,IF(MONTH(K18)&lt;10,10,IF(MONTH(K18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(K18),{2,4,5,6,7,8,10,12},0)),DAY(K18)&lt;=14),MONTH(K18),IF(MONTH(K18)&lt;2,2,IF(MONTH(K18)&lt;4,4,IF(MONTH(K18)&lt;8,MONTH(K18)+1,IF(MONTH(K18)&lt;10,10,IF(MONTH(K18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(K18),{2,4,5,6,7,8,10,12},0)),DAY(K18)&lt;=14),MONTH(K18),IF(MONTH(K18)&lt;2,2,IF(MONTH(K18)&lt;4,4,IF(MONTH(K18)&lt;8,MONTH(K18)+1,IF(MONTH(K18)&lt;10,10,IF(MONTH(K18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="20">
+        <f>(YEAR(L18)+(IF(AND(ISNUMBER(MATCH(MONTH(L18),{2,4,5,6,7,8,10,12},0)),DAY(L18)&lt;=14),MONTH(L18),IF(MONTH(L18)&lt;2,2,IF(MONTH(L18)&lt;4,4,IF(MONTH(L18)&lt;8,MONTH(L18)+1,IF(MONTH(L18)&lt;10,10,IF(MONTH(L18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(L18),{2,4,5,6,7,8,10,12},0)),DAY(L18)&lt;=14),MONTH(L18),IF(MONTH(L18)&lt;2,2,IF(MONTH(L18)&lt;4,4,IF(MONTH(L18)&lt;8,MONTH(L18)+1,IF(MONTH(L18)&lt;10,10,IF(MONTH(L18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(L18),{2,4,5,6,7,8,10,12},0)),DAY(L18)&lt;=14),MONTH(L18),IF(MONTH(L18)&lt;2,2,IF(MONTH(L18)&lt;4,4,IF(MONTH(L18)&lt;8,MONTH(L18)+1,IF(MONTH(L18)&lt;10,10,IF(MONTH(L18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+      <c r="M19" s="20">
+        <f>(YEAR(M18)+(IF(AND(ISNUMBER(MATCH(MONTH(M18),{2,4,5,6,7,8,10,12},0)),DAY(M18)&lt;=14),MONTH(M18),IF(MONTH(M18)&lt;2,2,IF(MONTH(M18)&lt;4,4,IF(MONTH(M18)&lt;8,MONTH(M18)+1,IF(MONTH(M18)&lt;10,10,IF(MONTH(M18)&lt;12,12,14))))))&gt;12))&amp;"-"&amp;TEXT(IF(AND(ISNUMBER(MATCH(MONTH(M18),{2,4,5,6,7,8,10,12},0)),DAY(M18)&lt;=14),MONTH(M18),IF(MONTH(M18)&lt;2,2,IF(MONTH(M18)&lt;4,4,IF(MONTH(M18)&lt;8,MONTH(M18)+1,IF(MONTH(M18)&lt;10,10,IF(MONTH(M18)&lt;12,12,14))))))-12*(IF(AND(ISNUMBER(MATCH(MONTH(M18),{2,4,5,6,7,8,10,12},0)),DAY(M18)&lt;=14),MONTH(M18),IF(MONTH(M18)&lt;2,2,IF(MONTH(M18)&lt;4,4,IF(MONTH(M18)&lt;8,MONTH(M18)+1,IF(MONTH(M18)&lt;10,10,IF(MONTH(M18)&lt;12,12,14))))))&gt;12),"00")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="B20" s="5">
+        <f>(B11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="C20" s="5">
+        <f>(C11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="D20" s="5">
+        <f>(D11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <f>(E11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <f>(F11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <f>(G11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="5">
+        <f>(H11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="5">
+        <f>(I11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="5">
+        <f>(J11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="5">
+        <f>(K11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="5">
+        <f>(L11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="M20" s="5">
+        <f>(M11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="B21" s="5">
+        <f>(B12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="5">
+        <f>(C12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="5">
+        <f>(D12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="5">
+        <f>(E12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <f>(F12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="5">
+        <f>(G12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="H21" s="5">
+        <f>(H12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="5">
+        <f>(I12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="5">
+        <f>(J12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="K21" s="5">
+        <f>(K12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="L21" s="5">
+        <f>(L12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+      <c r="M21" s="5">
+        <f>(M12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B22" s="5">
+        <f>B14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+B15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="5">
+        <f>C14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+C15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="5">
+        <f>D14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+D15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
+        <f>E14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+E15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <f>F14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+F15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <f>G14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+G15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="5">
+        <f>H14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+H15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="5">
+        <f>I14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+I15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="5">
+        <f>J14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+J15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="K22" s="5">
+        <f>K14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+K15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="L22" s="5">
+        <f>L14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+L15+Premium</f>
+        <v>0</v>
+      </c>
+      <c r="M22" s="5">
+        <f>M14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+M15+Premium</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
+      <c r="A23" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*B22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="C23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*C22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="D23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*D22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*E22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="F23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*F22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*G22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="H23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*H22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*I22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*J22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="K23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*K22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="L23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*L22/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="M23" s="5">
+        <f>HeadSold*CrWeight*YieldPct/100/100*M22/HeadSold</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="B24" s="5">
+        <f>HeadPlaced*(B10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="5">
+        <f>HeadPlaced*(C10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="5">
+        <f>HeadPlaced*(D10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="5">
+        <f>HeadPlaced*(E10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <f>HeadPlaced*(F10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
+        <f>HeadPlaced*(G10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="5">
+        <f>HeadPlaced*(H10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="5">
+        <f>HeadPlaced*(I10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="5">
+        <f>HeadPlaced*(J10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="5">
+        <f>HeadPlaced*(K10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="L24" s="5">
+        <f>HeadPlaced*(L10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="5">
+        <f>HeadPlaced*(M10+WeanAdder+WeanFreight)/HeadSold</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="B25" s="5">
+        <f>(FeedCornBu*B20+FeedSbmTons*B21+FeedDdgsTons*B13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="C25" s="5">
+        <f>(FeedCornBu*C20+FeedSbmTons*C21+FeedDdgsTons*C13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="5">
+        <f>(FeedCornBu*D20+FeedSbmTons*D21+FeedDdgsTons*D13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="5">
+        <f>(FeedCornBu*E20+FeedSbmTons*E21+FeedDdgsTons*E13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
+        <f>(FeedCornBu*F20+FeedSbmTons*F21+FeedDdgsTons*F13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="5">
+        <f>(FeedCornBu*G20+FeedSbmTons*G21+FeedDdgsTons*G13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="H25" s="5">
+        <f>(FeedCornBu*H20+FeedSbmTons*H21+FeedDdgsTons*H13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="5">
+        <f>(FeedCornBu*I20+FeedSbmTons*I21+FeedDdgsTons*I13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="5">
+        <f>(FeedCornBu*J20+FeedSbmTons*J21+FeedDdgsTons*J13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="K25" s="5">
+        <f>(FeedCornBu*K20+FeedSbmTons*K21+FeedDdgsTons*K13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="L25" s="5">
+        <f>(FeedCornBu*L20+FeedSbmTons*L21+FeedDdgsTons*L13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="M25" s="5">
+        <f>(FeedCornBu*M20+FeedSbmTons*M21+FeedDdgsTons*M13+FeedOtherUsd+FeedTons*FeedMill)/HeadSold</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="B26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="C26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="K26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="L26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="M26" s="5">
+        <f>IF(BarnMode="$/space/year",HeadPlaced*BarnRent*(CrDays+BarnDowntime)/365,HeadPlaced*BarnPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="B27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="K27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="L27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="5">
+        <f>(CostLabor+CostVet+CostUtilities+CostTrucking+CostInsMisc+CostGA+CostMortality+CostOther)/HeadSold</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="B28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(B10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*B20+FeedSbmTons*B21+FeedDdgsTons*B13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(C10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*C20+FeedSbmTons*C21+FeedDdgsTons*C13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(D10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*D20+FeedSbmTons*D21+FeedDdgsTons*D13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(E10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*E20+FeedSbmTons*E21+FeedDdgsTons*E13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(F10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*F20+FeedSbmTons*F21+FeedDdgsTons*F13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(G10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*G20+FeedSbmTons*G21+FeedDdgsTons*G13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(H10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*H20+FeedSbmTons*H21+FeedDdgsTons*H13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(I10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*I20+FeedSbmTons*I21+FeedDdgsTons*I13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(J10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*J20+FeedSbmTons*J21+FeedDdgsTons*J13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="K28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(K10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*K20+FeedSbmTons*K21+FeedDdgsTons*K13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="L28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(L10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*L20+FeedSbmTons*L21+FeedDdgsTons*L13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+      <c r="M28" s="5">
+        <f>IF(InterestMode="annual rate",InterestPct/100*CrDays/365*(HeadPlaced*(M10+WeanAdder+WeanFreight)+0.5*(FeedCornBu*M20+FeedSbmTons*M21+FeedDdgsTons*M13+FeedOtherUsd+FeedTons*FeedMill)),HeadPlaced*InterestPerPig)/HeadSold</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="B29" s="5">
+        <f>B23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="5">
+        <f>C23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="5">
+        <f>D23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="5">
+        <f>E23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="5">
+        <f>F23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="5">
+        <f>G23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="5">
+        <f>H23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="5">
+        <f>I23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="5">
+        <f>J23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="K29" s="5">
+        <f>K23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="L29" s="5">
+        <f>L23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+      <c r="M29" s="5">
+        <f>M23*CheckoffPct/100</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="B30" s="5">
+        <f>B24+B25+B26+B27+B28+B29</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="5">
+        <f>C24+C25+C26+C27+C28+C29</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="5">
+        <f>D24+D25+D26+D27+D28+D29</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="5">
+        <f>E24+E25+E26+E27+E28+E29</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="5">
+        <f>F24+F25+F26+F27+F28+F29</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="5">
+        <f>G24+G25+G26+G27+G28+G29</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="5">
+        <f>H24+H25+H26+H27+H28+H29</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="5">
+        <f>I24+I25+I26+I27+I28+I29</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="5">
+        <f>J24+J25+J26+J27+J28+J29</f>
+        <v>0</v>
+      </c>
+      <c r="K30" s="5">
+        <f>K24+K25+K26+K27+K28+K29</f>
+        <v>0</v>
+      </c>
+      <c r="L30" s="5">
+        <f>L24+L25+L26+L27+L28+L29</f>
+        <v>0</v>
+      </c>
+      <c r="M30" s="5">
+        <f>M24+M25+M26+M27+M28+M29</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="B31" s="5">
+        <f>B23-B30</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="5">
+        <f>C23-C30</f>
+        <v>0</v>
+      </c>
+      <c r="D31" s="5">
+        <f>D23-D30</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="5">
+        <f>E23-E30</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="5">
+        <f>F23-F30</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="5">
+        <f>G23-G30</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="5">
+        <f>H23-H30</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="5">
+        <f>I23-I30</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="5">
+        <f>J23-J30</f>
+        <v>0</v>
+      </c>
+      <c r="K31" s="5">
+        <f>K23-K30</f>
+        <v>0</v>
+      </c>
+      <c r="L31" s="5">
+        <f>L23-L30</f>
+        <v>0</v>
+      </c>
+      <c r="M31" s="5">
+        <f>M23-M30</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B32" s="5">
+        <f>B31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="5">
+        <f>C31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="5">
+        <f>D31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="5">
+        <f>E31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="5">
+        <f>F31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="5">
+        <f>G31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="5">
+        <f>H31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="5">
+        <f>I31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="5">
+        <f>J31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="K32" s="5">
+        <f>K31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="L32" s="5">
+        <f>L31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+      <c r="M32" s="5">
+        <f>M31-(Principal+TermInterest)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Third review: crush drops hedges, stale/future weeks, Barchart fixes
- Weekly crush (Python and Excel) leaves the group's hedges out.
- build_weeks: weeks after today use today's prices; stale as-of prices flagged.
- Barchart: corn cash vs futures kinds, grain eighths, cents on save,
  plausibility warnings, validated contract box; contract basis overlays
  the base history.
- App: hedged % without a price is a blocking problem; warn when a sale
  half-month has no basis history.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTSCZNmEoT9CgCPoTHxFfB
</commit_message>
<xml_diff>
--- a/W2F_Projection.xlsx
+++ b/W2F_Projection.xlsx
@@ -5765,51 +5765,51 @@
         <v>253</v>
       </c>
       <c r="B20" s="5">
-        <f>(B11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(B11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="C20" s="5">
-        <f>(C11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(C11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="D20" s="5">
-        <f>(D11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(D11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="E20" s="5">
-        <f>(E11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(E11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="F20" s="5">
-        <f>(F11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(F11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="G20" s="5">
-        <f>(G11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(G11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="H20" s="5">
-        <f>(H11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(H11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="I20" s="5">
-        <f>(I11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(I11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="J20" s="5">
-        <f>(J11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(J11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="K20" s="5">
-        <f>(K11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(K11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="L20" s="5">
-        <f>(L11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(L11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
       <c r="M20" s="5">
-        <f>(M11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)*(1-CornHedgePct/100)+CornHedged*CornHedgePct/100</f>
+        <f>(M11+IF(CrCornCash="Yes",0,CornBasis)+CornCarry)</f>
         <v>0</v>
       </c>
     </row>
@@ -5818,51 +5818,51 @@
         <v>254</v>
       </c>
       <c r="B21" s="5">
-        <f>(B12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>B12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="C21" s="5">
-        <f>(C12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>C12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="D21" s="5">
-        <f>(D12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>D12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="E21" s="5">
-        <f>(E12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>E12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="F21" s="5">
-        <f>(F12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>F12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="G21" s="5">
-        <f>(G12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>G12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="H21" s="5">
-        <f>(H12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>H12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="I21" s="5">
-        <f>(I12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>I12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="J21" s="5">
-        <f>(J12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>J12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="K21" s="5">
-        <f>(K12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>K12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="L21" s="5">
-        <f>(L12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>L12+SbmBasis</f>
         <v>0</v>
       </c>
       <c r="M21" s="5">
-        <f>(M12+SbmBasis)*(1-SbmHedgePct/100)+SbmHedged*SbmHedgePct/100</f>
+        <f>M12+SbmBasis</f>
         <v>0</v>
       </c>
     </row>
@@ -5871,51 +5871,51 @@
         <v>201</v>
       </c>
       <c r="B22" s="5">
-        <f>B14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+B15+Premium</f>
+        <f>B14+B15+Premium</f>
         <v>0</v>
       </c>
       <c r="C22" s="5">
-        <f>C14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+C15+Premium</f>
+        <f>C14+C15+Premium</f>
         <v>0</v>
       </c>
       <c r="D22" s="5">
-        <f>D14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+D15+Premium</f>
+        <f>D14+D15+Premium</f>
         <v>0</v>
       </c>
       <c r="E22" s="5">
-        <f>E14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+E15+Premium</f>
+        <f>E14+E15+Premium</f>
         <v>0</v>
       </c>
       <c r="F22" s="5">
-        <f>F14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+F15+Premium</f>
+        <f>F14+F15+Premium</f>
         <v>0</v>
       </c>
       <c r="G22" s="5">
-        <f>G14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+G15+Premium</f>
+        <f>G14+G15+Premium</f>
         <v>0</v>
       </c>
       <c r="H22" s="5">
-        <f>H14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+H15+Premium</f>
+        <f>H14+H15+Premium</f>
         <v>0</v>
       </c>
       <c r="I22" s="5">
-        <f>I14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+I15+Premium</f>
+        <f>I14+I15+Premium</f>
         <v>0</v>
       </c>
       <c r="J22" s="5">
-        <f>J14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+J15+Premium</f>
+        <f>J14+J15+Premium</f>
         <v>0</v>
       </c>
       <c r="K22" s="5">
-        <f>K14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+K15+Premium</f>
+        <f>K14+K15+Premium</f>
         <v>0</v>
       </c>
       <c r="L22" s="5">
-        <f>L14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+L15+Premium</f>
+        <f>L14+L15+Premium</f>
         <v>0</v>
       </c>
       <c r="M22" s="5">
-        <f>M14*(1-HogHedgePct/100)+HogHedged*HogHedgePct/100+M15+Premium</f>
+        <f>M14+M15+Premium</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>